<commit_message>
feat: atualizacoes e melhorias do sistema LeoOtica
</commit_message>
<xml_diff>
--- a/backend/teste_excel.xlsx
+++ b/backend/teste_excel.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,11 +73,17 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002A6BB8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="0078350F"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +110,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F9FAFB"/>
+        <bgColor rgb="00F9FAFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFBEB"/>
         <bgColor rgb="00FFFBEB"/>
       </patternFill>
@@ -240,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -279,17 +291,47 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -655,7 +697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I22"/>
+  <dimension ref="B2:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -713,7 +755,7 @@
     <row r="6">
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>#REQ-20260801-000</t>
+          <t>#REQ-20260809-015</t>
         </is>
       </c>
       <c r="C6" s="13" t="n"/>
@@ -735,7 +777,7 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>01/08/2026 15:57 (Horário de Brasília)</t>
+          <t>09/08/2026 23:15 (Horário de Brasília)</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -839,68 +881,698 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="21" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>LENS-156-BLO-001</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] Bloco Visão Simples Surfaçado Resina Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="G14" s="26" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I14" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>LENS-156-MUL-002</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>[LENTE] Multifocal Bloco Semi-Acabado Resina Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="G15" s="31" t="inlineStr">
+        <is>
+          <t>9 un</t>
+        </is>
+      </c>
+      <c r="H15" s="31" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I15" s="33" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>LENS-150-LP-003</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] LP Incolor 1.50 CR-39 Incolor Ø70mm</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
+      <c r="G16" s="26" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I16" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>LENS-156-LEN-004</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>[LENTE] Lente Pronta LP 1.56 Resina Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="inlineStr">
+        <is>
+          <t>-2.00</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>-0.50</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H17" s="31" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I17" s="33" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>LENS-156-MUL-005</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] Multifocal Bloco Semi-Acabado Resina Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="inlineStr">
+        <is>
+          <t>9 un</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I18" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>LENS-150-LP-006</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>[LENTE] LP Incolor 1.50 CR-39 Incolor Ø70mm</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H19" s="31" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I19" s="33" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>LENS-150-LP-007</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] LP Incolor 1.50 CR-39 Incolor Ø70mm</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>-3.50</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="inlineStr">
+        <is>
+          <t>-0.75</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I20" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>LENS-156-MUL-008</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>[LENTE] Multifocal Acabado Prog Resina Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E21" s="32" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="G21" s="31" t="inlineStr">
+        <is>
+          <t>9 un</t>
+        </is>
+      </c>
+      <c r="H21" s="31" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I21" s="33" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>LENS-156-GRA-009</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] Grade 1.67 Asférica Resina Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>-4.00</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="inlineStr">
+        <is>
+          <t>-1.50</t>
+        </is>
+      </c>
+      <c r="G22" s="26" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I22" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>LENS-156-MUL-010</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>[LENTE] Multifocal Acabado Prog Resina Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="inlineStr">
+        <is>
+          <t>9 un</t>
+        </is>
+      </c>
+      <c r="H23" s="31" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I23" s="33" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>LENS-156-VIS-011</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] Visão Simples LP 1.56 AR Resina 1.56 Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>-3.50</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
+      <c r="G24" s="26" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I24" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>LENS-150-LP-012</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>[LENTE] LP Incolor 1.50 CR-39 Incolor Ø70mm</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="E25" s="32" t="inlineStr">
+        <is>
+          <t>-3.50</t>
+        </is>
+      </c>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>-0.75</t>
+        </is>
+      </c>
+      <c r="G25" s="31" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H25" s="31" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I25" s="33" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>LENS-156-VIS-013</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] Visão Simples LP 1.56 AR Resina 1.56 Anti-Reflexo AR Ø70mm</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>-1.50</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="inlineStr">
+        <is>
+          <t>-0.50</t>
+        </is>
+      </c>
+      <c r="G26" s="26" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H26" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I26" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>LENS-150-LP-014</t>
+        </is>
+      </c>
+      <c r="C27" s="30" t="inlineStr">
+        <is>
+          <t>[LENTE] LP Incolor 1.50 CR-39 Incolor Ø70mm</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="E27" s="32" t="inlineStr">
+        <is>
+          <t>-3.50</t>
+        </is>
+      </c>
+      <c r="F27" s="32" t="inlineStr">
+        <is>
+          <t>-0.75</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H27" s="31" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I27" s="33" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>LENS-150-LP-015</t>
+        </is>
+      </c>
+      <c r="C28" s="25" t="inlineStr">
+        <is>
+          <t>[LENTE] LP Incolor 1.50 CR-39 Incolor Ø70mm</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
+      <c r="G28" s="26" t="inlineStr">
+        <is>
+          <t>8 un</t>
+        </is>
+      </c>
+      <c r="H28" s="26" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+      <c r="I28" s="28" t="inlineStr">
+        <is>
+          <t>0 un</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>Diretrizes de Logística e Transição de Estados</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="24" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="34" t="inlineStr">
         <is>
           <t>Nota Automática do Sistema:
 1. As dioptrias listadas acima atingiram ou ultrapassaram o limite crítico de ruptura (estoque abaixo do nível de segurança). Este lote foi projetado com base na taxa de consumo diário (daily_burn_rate) para suprir os próximos 15 dias de operação.
 2. Para evitar duplicidade de pedidos por gatilhos repetidos, as respectivas células da Grade Óptica foram alteradas temporariamente para o estado STATUS_AWAITING_SUPPLIER até a recepção física da nota de faturamento.</t>
         </is>
       </c>
-      <c r="C18" s="25" t="n"/>
-      <c r="D18" s="25" t="n"/>
-      <c r="E18" s="25" t="n"/>
-      <c r="F18" s="25" t="n"/>
-      <c r="G18" s="25" t="n"/>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="26" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="27" t="n"/>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="28" t="n"/>
-      <c r="E19" s="28" t="n"/>
-      <c r="F19" s="28" t="n"/>
-      <c r="G19" s="28" t="n"/>
-      <c r="H19" s="28" t="n"/>
-      <c r="I19" s="29" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="27" t="n"/>
-      <c r="C20" s="28" t="n"/>
-      <c r="D20" s="28" t="n"/>
-      <c r="E20" s="28" t="n"/>
-      <c r="F20" s="28" t="n"/>
-      <c r="G20" s="28" t="n"/>
-      <c r="H20" s="28" t="n"/>
-      <c r="I20" s="29" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="27" t="n"/>
-      <c r="C21" s="28" t="n"/>
-      <c r="D21" s="28" t="n"/>
-      <c r="E21" s="28" t="n"/>
-      <c r="F21" s="28" t="n"/>
-      <c r="G21" s="28" t="n"/>
-      <c r="H21" s="28" t="n"/>
-      <c r="I21" s="29" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="30" t="n"/>
-      <c r="C22" s="31" t="n"/>
-      <c r="D22" s="31" t="n"/>
-      <c r="E22" s="31" t="n"/>
-      <c r="F22" s="31" t="n"/>
-      <c r="G22" s="31" t="n"/>
-      <c r="H22" s="31" t="n"/>
-      <c r="I22" s="32" t="n"/>
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="35" t="n"/>
+      <c r="E33" s="35" t="n"/>
+      <c r="F33" s="35" t="n"/>
+      <c r="G33" s="35" t="n"/>
+      <c r="H33" s="35" t="n"/>
+      <c r="I33" s="36" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="37" t="n"/>
+      <c r="C34" s="38" t="n"/>
+      <c r="D34" s="38" t="n"/>
+      <c r="E34" s="38" t="n"/>
+      <c r="F34" s="38" t="n"/>
+      <c r="G34" s="38" t="n"/>
+      <c r="H34" s="38" t="n"/>
+      <c r="I34" s="39" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="37" t="n"/>
+      <c r="C35" s="38" t="n"/>
+      <c r="D35" s="38" t="n"/>
+      <c r="E35" s="38" t="n"/>
+      <c r="F35" s="38" t="n"/>
+      <c r="G35" s="38" t="n"/>
+      <c r="H35" s="38" t="n"/>
+      <c r="I35" s="39" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="37" t="n"/>
+      <c r="C36" s="38" t="n"/>
+      <c r="D36" s="38" t="n"/>
+      <c r="E36" s="38" t="n"/>
+      <c r="F36" s="38" t="n"/>
+      <c r="G36" s="38" t="n"/>
+      <c r="H36" s="38" t="n"/>
+      <c r="I36" s="39" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="40" t="n"/>
+      <c r="C37" s="41" t="n"/>
+      <c r="D37" s="41" t="n"/>
+      <c r="E37" s="41" t="n"/>
+      <c r="F37" s="41" t="n"/>
+      <c r="G37" s="41" t="n"/>
+      <c r="H37" s="41" t="n"/>
+      <c r="I37" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -908,15 +1580,15 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="G2:I3"/>
     <mergeCell ref="C7:D7"/>
+    <mergeCell ref="B33:I37"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="B11:I11"/>
-    <mergeCell ref="B16:I16"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="G8:I8"/>
+    <mergeCell ref="B31:I31"/>
     <mergeCell ref="F5:I5"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B18:I22"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F6:I6"/>
   </mergeCells>

</xml_diff>